<commit_message>
Fix errors in project Gantt chart
Update the project schedule after correcting the chart
</commit_message>
<xml_diff>
--- a/IT-353 Project Gantt Chart.xlsx.xlsx
+++ b/IT-353 Project Gantt Chart.xlsx.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\osama\OneDrive\سطح المكتب\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9981D597-B0D4-4C51-8F28-B60415BFA03C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FC85280-BF18-401F-81E3-E91D88DF43F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -904,7 +904,7 @@
       <c r="AA9" s="3"/>
       <c r="AB9" s="10"/>
     </row>
-    <row r="10" spans="1:28" ht="18.649999999999999" customHeight="1">
+    <row r="10" spans="1:28" ht="25.5" customHeight="1">
       <c r="A10" s="9" t="s">
         <v>25</v>
       </c>
@@ -932,7 +932,7 @@
       <c r="AA10" s="3"/>
       <c r="AB10" s="10"/>
     </row>
-    <row r="11" spans="1:28" ht="18.5" customHeight="1">
+    <row r="11" spans="1:28" ht="38" customHeight="1">
       <c r="A11" s="9" t="s">
         <v>27</v>
       </c>
@@ -960,7 +960,7 @@
       <c r="AA11" s="3"/>
       <c r="AB11" s="10"/>
     </row>
-    <row r="12" spans="1:28" ht="18.649999999999999" customHeight="1">
+    <row r="12" spans="1:28" ht="38.5" customHeight="1">
       <c r="A12" s="9" t="s">
         <v>29</v>
       </c>

</xml_diff>